<commit_message>
Nothing to note, just a cleaning update
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/order_archive/Performance Food/Performance Food_Bakery_20260714.xlsx
+++ b/WorkBot/main/data/order_archive/Performance Food/Performance Food_Bakery_20260714.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,6 +521,405 @@
         <v>38.7</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FL098</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sugar - Extra Fine</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>29.79</v>
+      </c>
+      <c r="E8" t="n">
+        <v>178.74</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>G5010</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carrots - Jumbo Fresh</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>42.51</v>
+      </c>
+      <c r="E9" t="n">
+        <v>42.51</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HB946</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Peppers - Banana</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>31.33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>31.33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T0948</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Almond Milk</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>35.74</v>
+      </c>
+      <c r="E11" t="n">
+        <v>35.74</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BEH52</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Joe Tea - Raspberry</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E12" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AKH94</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Joe Tea - Mango Lemonade</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E13" t="n">
+        <v>43.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AKH96</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Joe Tea - Lemon</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E14" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AKW10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Joe Tea - Kiwi Strawberry</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E15" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AKJ04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Joe Tea - Black Unsweetened</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E16" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>H2822</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cannoli Shells - Large</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>34.17</v>
+      </c>
+      <c r="E17" t="n">
+        <v>102.51</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10198</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Capers</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>69.20999999999999</v>
+      </c>
+      <c r="E18" t="n">
+        <v>69.20999999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MN198</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tuna - Ahi (Sesame Seared)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>174.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>174.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VF610</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Joyba Bubble Tea - Mango Passion Fruit</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="E20" t="n">
+        <v>54.52</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VF608</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Joyba Bubble Tea - Green Strawberry Lemonade</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="E21" t="n">
+        <v>55.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CM230</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Oat Milk</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>15</v>
+      </c>
+      <c r="D22" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="E22" t="n">
+        <v>234.75</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WF580</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Corned Beef (Sliced)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>71.20999999999999</v>
+      </c>
+      <c r="E23" t="n">
+        <v>213.63</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>34768</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Potato - Red Large (A)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>20.48</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>K1570</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Buttermilk</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="E25" t="n">
+        <v>36.76</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FB270</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roma - Tiramisu Plastic Cup</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>34.79</v>
+      </c>
+      <c r="E26" t="n">
+        <v>34.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>